<commit_message>
Sheet: regenerate to show bac/sterile water; fix NAD+ 1000mg $265->$260; add NAD+ to catalog
- static/price_list.xlsx was stale (predated the water rows) — regenerated so the
  sent sheet now shows Bacteriostatic + Sterile Water ($12).
- NAD+ 1000mg corrected $265 -> $260 on the sheet.
- NAD+ added to pricing catalog (100mg $100 / 500mg $240 / 1000mg $260) so the agent
  quotes it from the sheet instead of improvising.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/price_list.xlsx
+++ b/static/price_list.xlsx
@@ -761,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2338,176 +2338,176 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="4" t="inlineStr">
+    <row r="75" ht="16" customHeight="1">
+      <c r="A75" s="41" t="inlineStr">
+        <is>
+          <t>BAC10</t>
+        </is>
+      </c>
+      <c r="B75" s="42" t="inlineStr">
+        <is>
+          <t>Bacteriostatic Water</t>
+        </is>
+      </c>
+      <c r="C75" s="43" t="inlineStr">
+        <is>
+          <t>10ml</t>
+        </is>
+      </c>
+      <c r="D75" s="44" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="16" customHeight="1">
+      <c r="A76" s="45" t="inlineStr">
+        <is>
+          <t>STW10</t>
+        </is>
+      </c>
+      <c r="B76" s="46" t="inlineStr">
+        <is>
+          <t>Sterile Water</t>
+        </is>
+      </c>
+      <c r="C76" s="47" t="inlineStr">
+        <is>
+          <t>10ml</t>
+        </is>
+      </c>
+      <c r="D76" s="48" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>生长激素  (GH / GROWTH)</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="16" customHeight="1">
-      <c r="A76" s="41" t="inlineStr">
+    <row r="78" ht="16" customHeight="1">
+      <c r="A78" s="49" t="inlineStr">
         <is>
           <t>IP2</t>
         </is>
       </c>
-      <c r="B76" s="42" t="inlineStr">
+      <c r="B78" s="50" t="inlineStr">
         <is>
           <t>Ipamorelin</t>
         </is>
       </c>
-      <c r="C76" s="43" t="inlineStr">
+      <c r="C78" s="51" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D76" s="44" t="inlineStr">
+      <c r="D78" s="52" t="inlineStr">
         <is>
           <t>$47</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="16" customHeight="1">
-      <c r="A77" s="41" t="inlineStr">
+    <row r="79" ht="16" customHeight="1">
+      <c r="A79" s="49" t="inlineStr">
         <is>
           <t>IP5</t>
         </is>
       </c>
-      <c r="B77" s="42" t="inlineStr">
+      <c r="B79" s="50" t="inlineStr">
         <is>
           <t>Ipamorelin</t>
         </is>
       </c>
-      <c r="C77" s="43" t="inlineStr">
+      <c r="C79" s="51" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D77" s="44" t="inlineStr">
+      <c r="D79" s="52" t="inlineStr">
         <is>
           <t>$58</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="16" customHeight="1">
-      <c r="A78" s="41" t="inlineStr">
+    <row r="80" ht="16" customHeight="1">
+      <c r="A80" s="49" t="inlineStr">
         <is>
           <t>IP10</t>
         </is>
       </c>
-      <c r="B78" s="42" t="inlineStr">
+      <c r="B80" s="50" t="inlineStr">
         <is>
           <t>Ipamorelin</t>
         </is>
       </c>
-      <c r="C78" s="43" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D78" s="44" t="inlineStr">
+      <c r="C80" s="51" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D80" s="52" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="45" t="inlineStr">
+    <row r="81" ht="16" customHeight="1">
+      <c r="A81" s="53" t="inlineStr">
         <is>
           <t>CND2</t>
         </is>
       </c>
-      <c r="B79" s="46" t="inlineStr">
+      <c r="B81" s="54" t="inlineStr">
         <is>
           <t>CJC-1295 (no DAC)</t>
         </is>
       </c>
-      <c r="C79" s="47" t="inlineStr">
+      <c r="C81" s="55" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D79" s="48" t="inlineStr">
+      <c r="D81" s="56" t="inlineStr">
         <is>
           <t>$42</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="45" t="inlineStr">
+    <row r="82" ht="16" customHeight="1">
+      <c r="A82" s="53" t="inlineStr">
         <is>
           <t>CND5</t>
         </is>
       </c>
-      <c r="B80" s="46" t="inlineStr">
+      <c r="B82" s="54" t="inlineStr">
         <is>
           <t>CJC-1295 (no DAC)</t>
         </is>
       </c>
-      <c r="C80" s="47" t="inlineStr">
+      <c r="C82" s="55" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D80" s="48" t="inlineStr">
+      <c r="D82" s="56" t="inlineStr">
         <is>
           <t>$98</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="45" t="inlineStr">
-        <is>
-          <t>CND10</t>
-        </is>
-      </c>
-      <c r="B81" s="46" t="inlineStr">
-        <is>
-          <t>CJC-1295 (no DAC)</t>
-        </is>
-      </c>
-      <c r="C81" s="47" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D81" s="48" t="inlineStr">
-        <is>
-          <t>$158</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="16" customHeight="1">
-      <c r="A82" s="49" t="inlineStr">
-        <is>
-          <t>CD5</t>
-        </is>
-      </c>
-      <c r="B82" s="50" t="inlineStr">
-        <is>
-          <t>CJC-1295 (w/ DAC)</t>
-        </is>
-      </c>
-      <c r="C82" s="51" t="inlineStr">
-        <is>
-          <t>5mg</t>
-        </is>
-      </c>
-      <c r="D82" s="52" t="inlineStr">
-        <is>
-          <t>$166</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="53" t="inlineStr">
         <is>
-          <t>CP10</t>
+          <t>CND10</t>
         </is>
       </c>
       <c r="B83" s="54" t="inlineStr">
         <is>
-          <t>CJC+Ipa Blend</t>
+          <t>CJC-1295 (no DAC)</t>
         </is>
       </c>
       <c r="C83" s="55" t="inlineStr">
@@ -2517,437 +2517,437 @@
       </c>
       <c r="D83" s="56" t="inlineStr">
         <is>
-          <t>$114</t>
+          <t>$158</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="57" t="inlineStr">
         <is>
+          <t>CD5</t>
+        </is>
+      </c>
+      <c r="B84" s="58" t="inlineStr">
+        <is>
+          <t>CJC-1295 (w/ DAC)</t>
+        </is>
+      </c>
+      <c r="C84" s="59" t="inlineStr">
+        <is>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D84" s="60" t="inlineStr">
+        <is>
+          <t>$166</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="16" customHeight="1">
+      <c r="A85" s="61" t="inlineStr">
+        <is>
+          <t>CP10</t>
+        </is>
+      </c>
+      <c r="B85" s="62" t="inlineStr">
+        <is>
+          <t>CJC+Ipa Blend</t>
+        </is>
+      </c>
+      <c r="C85" s="63" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D85" s="64" t="inlineStr">
+        <is>
+          <t>$114</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="65" t="inlineStr">
+        <is>
           <t>SMO5</t>
         </is>
       </c>
-      <c r="B84" s="58" t="inlineStr">
+      <c r="B86" s="66" t="inlineStr">
         <is>
           <t>Sermorelin</t>
         </is>
       </c>
-      <c r="C84" s="59" t="inlineStr">
+      <c r="C86" s="67" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D84" s="60" t="inlineStr">
+      <c r="D86" s="68" t="inlineStr">
         <is>
           <t>$90</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="16" customHeight="1">
-      <c r="A85" s="57" t="inlineStr">
+    <row r="87" ht="16" customHeight="1">
+      <c r="A87" s="65" t="inlineStr">
         <is>
           <t>SMO10</t>
         </is>
       </c>
-      <c r="B85" s="58" t="inlineStr">
+      <c r="B87" s="66" t="inlineStr">
         <is>
           <t>Sermorelin</t>
         </is>
       </c>
-      <c r="C85" s="59" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D85" s="60" t="inlineStr">
+      <c r="C87" s="67" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D87" s="68" t="inlineStr">
         <is>
           <t>$119</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="16" customHeight="1">
-      <c r="A86" s="61" t="inlineStr">
+    <row r="88" ht="16" customHeight="1">
+      <c r="A88" s="5" t="inlineStr">
         <is>
           <t>G25</t>
         </is>
       </c>
-      <c r="B86" s="62" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>GHRP-2</t>
         </is>
       </c>
-      <c r="C86" s="63" t="inlineStr">
+      <c r="C88" s="7" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D86" s="64" t="inlineStr">
+      <c r="D88" s="8" t="inlineStr">
         <is>
           <t>$34</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="16" customHeight="1">
-      <c r="A87" s="61" t="inlineStr">
+    <row r="89" ht="16" customHeight="1">
+      <c r="A89" s="5" t="inlineStr">
         <is>
           <t>G210</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>GHRP-2</t>
         </is>
       </c>
-      <c r="C87" s="63" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D87" s="64" t="inlineStr">
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>$58</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="16" customHeight="1">
-      <c r="A88" s="65" t="inlineStr">
+    <row r="90" ht="16" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
         <is>
           <t>G65</t>
         </is>
       </c>
-      <c r="B88" s="66" t="inlineStr">
+      <c r="B90" s="10" t="inlineStr">
         <is>
           <t>GHRP-6</t>
         </is>
       </c>
-      <c r="C88" s="67" t="inlineStr">
+      <c r="C90" s="11" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D88" s="68" t="inlineStr">
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>$38</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="16" customHeight="1">
-      <c r="A89" s="65" t="inlineStr">
+    <row r="91" ht="16" customHeight="1">
+      <c r="A91" s="9" t="inlineStr">
         <is>
           <t>G610</t>
         </is>
       </c>
-      <c r="B89" s="66" t="inlineStr">
+      <c r="B91" s="10" t="inlineStr">
         <is>
           <t>GHRP-6</t>
         </is>
       </c>
-      <c r="C89" s="67" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D89" s="68" t="inlineStr">
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
         <is>
           <t>$42</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
+    <row r="92" ht="16" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
         <is>
           <t>HX2</t>
         </is>
       </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="B92" s="14" t="inlineStr">
         <is>
           <t>Hexarelin</t>
         </is>
       </c>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="C92" s="15" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D90" s="8" t="inlineStr">
+      <c r="D92" s="16" t="inlineStr">
         <is>
           <t>$56</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="16" customHeight="1">
-      <c r="A91" s="5" t="inlineStr">
+    <row r="93" ht="16" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
         <is>
           <t>HX5</t>
         </is>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B93" s="14" t="inlineStr">
         <is>
           <t>Hexarelin</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C93" s="15" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D91" s="8" t="inlineStr">
+      <c r="D93" s="16" t="inlineStr">
         <is>
           <t>$104</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="16" customHeight="1">
-      <c r="A92" s="9" t="inlineStr">
+    <row r="94" ht="16" customHeight="1">
+      <c r="A94" s="17" t="inlineStr">
         <is>
           <t>KS5</t>
         </is>
       </c>
-      <c r="B92" s="10" t="inlineStr">
+      <c r="B94" s="18" t="inlineStr">
         <is>
           <t>KissPeptin-10</t>
         </is>
       </c>
-      <c r="C92" s="11" t="inlineStr">
+      <c r="C94" s="19" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D92" s="12" t="inlineStr">
+      <c r="D94" s="20" t="inlineStr">
         <is>
           <t>$72</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="16" customHeight="1">
-      <c r="A93" s="9" t="inlineStr">
-        <is>
-          <t>KS10</t>
-        </is>
-      </c>
-      <c r="B93" s="10" t="inlineStr">
-        <is>
-          <t>KissPeptin-10</t>
-        </is>
-      </c>
-      <c r="C93" s="11" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D93" s="12" t="inlineStr">
-        <is>
-          <t>$116</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="16" customHeight="1">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>FM2</t>
-        </is>
-      </c>
-      <c r="B94" s="14" t="inlineStr">
-        <is>
-          <t>MGF</t>
-        </is>
-      </c>
-      <c r="C94" s="15" t="inlineStr">
-        <is>
-          <t>2mg</t>
-        </is>
-      </c>
-      <c r="D94" s="16" t="inlineStr">
-        <is>
-          <t>$58</t>
         </is>
       </c>
     </row>
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="17" t="inlineStr">
         <is>
-          <t>FMP2</t>
+          <t>KS10</t>
         </is>
       </c>
       <c r="B95" s="18" t="inlineStr">
         <is>
-          <t>PEG MGF</t>
+          <t>KissPeptin-10</t>
         </is>
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>2mg</t>
+          <t>10mg</t>
         </is>
       </c>
       <c r="D95" s="20" t="inlineStr">
         <is>
-          <t>$101</t>
+          <t>$116</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="21" t="inlineStr">
         <is>
+          <t>FM2</t>
+        </is>
+      </c>
+      <c r="B96" s="22" t="inlineStr">
+        <is>
+          <t>MGF</t>
+        </is>
+      </c>
+      <c r="C96" s="23" t="inlineStr">
+        <is>
+          <t>2mg</t>
+        </is>
+      </c>
+      <c r="D96" s="24" t="inlineStr">
+        <is>
+          <t>$58</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="16" customHeight="1">
+      <c r="A97" s="25" t="inlineStr">
+        <is>
+          <t>FMP2</t>
+        </is>
+      </c>
+      <c r="B97" s="26" t="inlineStr">
+        <is>
+          <t>PEG MGF</t>
+        </is>
+      </c>
+      <c r="C97" s="27" t="inlineStr">
+        <is>
+          <t>2mg</t>
+        </is>
+      </c>
+      <c r="D97" s="28" t="inlineStr">
+        <is>
+          <t>$101</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="16" customHeight="1">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
           <t>H8</t>
         </is>
       </c>
-      <c r="B96" s="22" t="inlineStr">
+      <c r="B98" s="30" t="inlineStr">
         <is>
           <t>HGH 191AA</t>
         </is>
       </c>
-      <c r="C96" s="23" t="inlineStr">
+      <c r="C98" s="31" t="inlineStr">
         <is>
           <t>8iu</t>
         </is>
       </c>
-      <c r="D96" s="24" t="inlineStr">
+      <c r="D98" s="32" t="inlineStr">
         <is>
           <t>$65</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="16" customHeight="1">
-      <c r="A97" s="21" t="inlineStr">
+    <row r="99" ht="16" customHeight="1">
+      <c r="A99" s="29" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
       </c>
-      <c r="B97" s="22" t="inlineStr">
+      <c r="B99" s="30" t="inlineStr">
         <is>
           <t>HGH 191AA</t>
         </is>
       </c>
-      <c r="C97" s="23" t="inlineStr">
+      <c r="C99" s="31" t="inlineStr">
         <is>
           <t>10iu</t>
         </is>
       </c>
-      <c r="D97" s="24" t="inlineStr">
+      <c r="D99" s="32" t="inlineStr">
         <is>
           <t>$80</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="16" customHeight="1">
-      <c r="A98" s="21" t="inlineStr">
+    <row r="100" ht="16" customHeight="1">
+      <c r="A100" s="29" t="inlineStr">
         <is>
           <t>H15</t>
         </is>
       </c>
-      <c r="B98" s="22" t="inlineStr">
+      <c r="B100" s="30" t="inlineStr">
         <is>
           <t>HGH 191AA</t>
         </is>
       </c>
-      <c r="C98" s="23" t="inlineStr">
+      <c r="C100" s="31" t="inlineStr">
         <is>
           <t>15iu</t>
         </is>
       </c>
-      <c r="D98" s="24" t="inlineStr">
+      <c r="D100" s="32" t="inlineStr">
         <is>
           <t>$106</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="16" customHeight="1">
-      <c r="A99" s="25" t="inlineStr">
+    <row r="101" ht="16" customHeight="1">
+      <c r="A101" s="33" t="inlineStr">
         <is>
           <t>G5K</t>
         </is>
       </c>
-      <c r="B99" s="26" t="inlineStr">
+      <c r="B101" s="34" t="inlineStr">
         <is>
           <t>HCG</t>
         </is>
       </c>
-      <c r="C99" s="27" t="inlineStr">
+      <c r="C101" s="35" t="inlineStr">
         <is>
           <t>5000IU</t>
         </is>
       </c>
-      <c r="D99" s="28" t="inlineStr">
+      <c r="D101" s="36" t="inlineStr">
         <is>
           <t>$104</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="16" customHeight="1">
-      <c r="A100" s="25" t="inlineStr">
-        <is>
-          <t>G10K</t>
-        </is>
-      </c>
-      <c r="B100" s="26" t="inlineStr">
-        <is>
-          <t>HCG</t>
-        </is>
-      </c>
-      <c r="C100" s="27" t="inlineStr">
-        <is>
-          <t>10000IU</t>
-        </is>
-      </c>
-      <c r="D100" s="28" t="inlineStr">
-        <is>
-          <t>$164</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="16" customHeight="1">
-      <c r="A101" s="29" t="inlineStr">
-        <is>
-          <t>IG1</t>
-        </is>
-      </c>
-      <c r="B101" s="30" t="inlineStr">
-        <is>
-          <t>IGF-1 LR3</t>
-        </is>
-      </c>
-      <c r="C101" s="31" t="inlineStr">
-        <is>
-          <t>1mg</t>
-        </is>
-      </c>
-      <c r="D101" s="32" t="inlineStr">
-        <is>
-          <t>$204</t>
         </is>
       </c>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="33" t="inlineStr">
         <is>
-          <t>IGD</t>
+          <t>G10K</t>
         </is>
       </c>
       <c r="B102" s="34" t="inlineStr">
         <is>
-          <t>IGF-DES</t>
+          <t>HCG</t>
         </is>
       </c>
       <c r="C102" s="35" t="inlineStr">
         <is>
-          <t>2mg</t>
+          <t>10000IU</t>
         </is>
       </c>
       <c r="D102" s="36" t="inlineStr">
         <is>
-          <t>$77</t>
+          <t>$164</t>
         </is>
       </c>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="37" t="inlineStr">
         <is>
-          <t>FN1</t>
+          <t>IG1</t>
         </is>
       </c>
       <c r="B103" s="38" t="inlineStr">
         <is>
-          <t>Follistatin</t>
+          <t>IGF-1 LR3</t>
         </is>
       </c>
       <c r="C103" s="39" t="inlineStr">
@@ -2957,1251 +2957,1295 @@
       </c>
       <c r="D103" s="40" t="inlineStr">
         <is>
-          <t>$290</t>
+          <t>$204</t>
         </is>
       </c>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="41" t="inlineStr">
         <is>
-          <t>AE1</t>
+          <t>IGD</t>
         </is>
       </c>
       <c r="B104" s="42" t="inlineStr">
         <is>
-          <t>ACE-031</t>
+          <t>IGF-DES</t>
         </is>
       </c>
       <c r="C104" s="43" t="inlineStr">
         <is>
-          <t>1mg</t>
+          <t>2mg</t>
         </is>
       </c>
       <c r="D104" s="44" t="inlineStr">
         <is>
-          <t>$243</t>
+          <t>$77</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="45" t="inlineStr">
         <is>
-          <t>TY10</t>
+          <t>FN1</t>
         </is>
       </c>
       <c r="B105" s="46" t="inlineStr">
         <is>
-          <t>Thymalin</t>
+          <t>Follistatin</t>
         </is>
       </c>
       <c r="C105" s="47" t="inlineStr">
         <is>
-          <t>10mg</t>
+          <t>1mg</t>
         </is>
       </c>
       <c r="D105" s="48" t="inlineStr">
         <is>
-          <t>$77</t>
+          <t>$290</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="49" t="inlineStr">
         <is>
+          <t>AE1</t>
+        </is>
+      </c>
+      <c r="B106" s="50" t="inlineStr">
+        <is>
+          <t>ACE-031</t>
+        </is>
+      </c>
+      <c r="C106" s="51" t="inlineStr">
+        <is>
+          <t>1mg</t>
+        </is>
+      </c>
+      <c r="D106" s="52" t="inlineStr">
+        <is>
+          <t>$243</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="16" customHeight="1">
+      <c r="A107" s="53" t="inlineStr">
+        <is>
+          <t>TY10</t>
+        </is>
+      </c>
+      <c r="B107" s="54" t="inlineStr">
+        <is>
+          <t>Thymalin</t>
+        </is>
+      </c>
+      <c r="C107" s="55" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D107" s="56" t="inlineStr">
+        <is>
+          <t>$77</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="16" customHeight="1">
+      <c r="A108" s="57" t="inlineStr">
+        <is>
           <t>TSM2</t>
         </is>
       </c>
-      <c r="B106" s="50" t="inlineStr">
+      <c r="B108" s="58" t="inlineStr">
         <is>
           <t>Tesamorelin</t>
         </is>
       </c>
-      <c r="C106" s="51" t="inlineStr">
+      <c r="C108" s="59" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D106" s="52" t="inlineStr">
+      <c r="D108" s="60" t="inlineStr">
         <is>
           <t>$72</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="16" customHeight="1">
-      <c r="A107" s="49" t="inlineStr">
+    <row r="109" ht="16" customHeight="1">
+      <c r="A109" s="57" t="inlineStr">
         <is>
           <t>TSM5</t>
         </is>
       </c>
-      <c r="B107" s="50" t="inlineStr">
+      <c r="B109" s="58" t="inlineStr">
         <is>
           <t>Tesamorelin</t>
         </is>
       </c>
-      <c r="C107" s="51" t="inlineStr">
+      <c r="C109" s="59" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D107" s="52" t="inlineStr">
+      <c r="D109" s="60" t="inlineStr">
         <is>
           <t>$115</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="16" customHeight="1">
-      <c r="A108" s="49" t="inlineStr">
+    <row r="110" ht="16" customHeight="1">
+      <c r="A110" s="57" t="inlineStr">
         <is>
           <t>TSM10</t>
         </is>
       </c>
-      <c r="B108" s="50" t="inlineStr">
+      <c r="B110" s="58" t="inlineStr">
         <is>
           <t>Tesamorelin</t>
         </is>
       </c>
-      <c r="C108" s="51" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D108" s="52" t="inlineStr">
+      <c r="C110" s="59" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D110" s="60" t="inlineStr">
         <is>
           <t>$195</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="16" customHeight="1">
-      <c r="A109" s="49" t="inlineStr">
-        <is>
-          <t>TSM20</t>
-        </is>
-      </c>
-      <c r="B109" s="50" t="inlineStr">
-        <is>
-          <t>Tesamorelin</t>
-        </is>
-      </c>
-      <c r="C109" s="51" t="inlineStr">
-        <is>
-          <t>20mg</t>
-        </is>
-      </c>
-      <c r="D109" s="52" t="inlineStr">
-        <is>
-          <t>$290</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="16" customHeight="1">
-      <c r="A110" s="53" t="inlineStr">
-        <is>
-          <t>ACTH5</t>
-        </is>
-      </c>
-      <c r="B110" s="54" t="inlineStr">
-        <is>
-          <t>ACTH</t>
-        </is>
-      </c>
-      <c r="C110" s="55" t="inlineStr">
-        <is>
-          <t>5mg</t>
-        </is>
-      </c>
-      <c r="D110" s="56" t="inlineStr">
-        <is>
-          <t>$183</t>
         </is>
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="57" t="inlineStr">
         <is>
+          <t>TSM20</t>
+        </is>
+      </c>
+      <c r="B111" s="58" t="inlineStr">
+        <is>
+          <t>Tesamorelin</t>
+        </is>
+      </c>
+      <c r="C111" s="59" t="inlineStr">
+        <is>
+          <t>20mg</t>
+        </is>
+      </c>
+      <c r="D111" s="60" t="inlineStr">
+        <is>
+          <t>$290</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="16" customHeight="1">
+      <c r="A112" s="61" t="inlineStr">
+        <is>
+          <t>ACTH5</t>
+        </is>
+      </c>
+      <c r="B112" s="62" t="inlineStr">
+        <is>
+          <t>ACTH</t>
+        </is>
+      </c>
+      <c r="C112" s="63" t="inlineStr">
+        <is>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D112" s="64" t="inlineStr">
+        <is>
+          <t>$183</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="16" customHeight="1">
+      <c r="A113" s="65" t="inlineStr">
+        <is>
           <t>EP0</t>
         </is>
       </c>
-      <c r="B111" s="58" t="inlineStr">
+      <c r="B113" s="66" t="inlineStr">
         <is>
           <t>EPO</t>
         </is>
       </c>
-      <c r="C111" s="59" t="inlineStr">
+      <c r="C113" s="67" t="inlineStr">
         <is>
           <t>3000IU</t>
         </is>
       </c>
-      <c r="D111" s="60" t="inlineStr">
+      <c r="D113" s="68" t="inlineStr">
         <is>
           <t>$149</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="4" t="inlineStr">
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>认知健康  (COGNITIVE &amp; WELLNESS)</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="16" customHeight="1">
-      <c r="A113" s="61" t="inlineStr">
+    <row r="115" ht="16" customHeight="1">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t>NJ100</t>
         </is>
       </c>
-      <c r="B113" s="62" t="inlineStr">
+      <c r="B115" s="6" t="inlineStr">
         <is>
           <t>NAD</t>
         </is>
       </c>
-      <c r="C113" s="63" t="inlineStr">
+      <c r="C115" s="7" t="inlineStr">
         <is>
           <t>100mg</t>
         </is>
       </c>
-      <c r="D113" s="64" t="inlineStr">
+      <c r="D115" s="8" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="16" customHeight="1">
-      <c r="A114" s="61" t="inlineStr">
+    <row r="116" ht="16" customHeight="1">
+      <c r="A116" s="5" t="inlineStr">
         <is>
           <t>NJ500</t>
         </is>
       </c>
-      <c r="B114" s="62" t="inlineStr">
+      <c r="B116" s="6" t="inlineStr">
         <is>
           <t>NAD</t>
         </is>
       </c>
-      <c r="C114" s="63" t="inlineStr">
+      <c r="C116" s="7" t="inlineStr">
         <is>
           <t>500mg</t>
         </is>
       </c>
-      <c r="D114" s="64" t="inlineStr">
+      <c r="D116" s="8" t="inlineStr">
         <is>
           <t>$240</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="16" customHeight="1">
-      <c r="A115" s="61" t="inlineStr">
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="5" t="inlineStr">
         <is>
           <t>NJ1000</t>
         </is>
       </c>
-      <c r="B115" s="62" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>NAD</t>
         </is>
       </c>
-      <c r="C115" s="63" t="inlineStr">
+      <c r="C117" s="7" t="inlineStr">
         <is>
           <t>1000mg</t>
         </is>
       </c>
-      <c r="D115" s="64" t="inlineStr">
-        <is>
-          <t>$265</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="16" customHeight="1">
-      <c r="A116" s="65" t="inlineStr">
+      <c r="D117" s="8" t="inlineStr">
+        <is>
+          <t>$260</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="A118" s="9" t="inlineStr">
         <is>
           <t>GTT4</t>
         </is>
       </c>
-      <c r="B116" s="66" t="inlineStr">
+      <c r="B118" s="10" t="inlineStr">
         <is>
           <t>Glutathione</t>
         </is>
       </c>
-      <c r="C116" s="67" t="inlineStr">
+      <c r="C118" s="11" t="inlineStr">
         <is>
           <t>400mg</t>
         </is>
       </c>
-      <c r="D116" s="68" t="inlineStr">
+      <c r="D118" s="12" t="inlineStr">
         <is>
           <t>$67</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="16" customHeight="1">
-      <c r="A117" s="65" t="inlineStr">
+    <row r="119" ht="16" customHeight="1">
+      <c r="A119" s="9" t="inlineStr">
         <is>
           <t>GTT</t>
         </is>
       </c>
-      <c r="B117" s="66" t="inlineStr">
+      <c r="B119" s="10" t="inlineStr">
         <is>
           <t>Glutathione</t>
         </is>
       </c>
-      <c r="C117" s="67" t="inlineStr">
+      <c r="C119" s="11" t="inlineStr">
         <is>
           <t>600mg</t>
         </is>
       </c>
-      <c r="D117" s="68" t="inlineStr">
+      <c r="D119" s="12" t="inlineStr">
         <is>
           <t>$87</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="16" customHeight="1">
-      <c r="A118" s="65" t="inlineStr">
+    <row r="120" ht="16" customHeight="1">
+      <c r="A120" s="9" t="inlineStr">
         <is>
           <t>GTT15</t>
         </is>
       </c>
-      <c r="B118" s="66" t="inlineStr">
+      <c r="B120" s="10" t="inlineStr">
         <is>
           <t>Glutathione</t>
         </is>
       </c>
-      <c r="C118" s="67" t="inlineStr">
+      <c r="C120" s="11" t="inlineStr">
         <is>
           <t>1500mg</t>
         </is>
       </c>
-      <c r="D118" s="68" t="inlineStr">
+      <c r="D120" s="12" t="inlineStr">
         <is>
           <t>$166</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="16" customHeight="1">
-      <c r="A119" s="5" t="inlineStr">
+    <row r="121" ht="16" customHeight="1">
+      <c r="A121" s="13" t="inlineStr">
         <is>
           <t>ET10</t>
         </is>
       </c>
-      <c r="B119" s="6" t="inlineStr">
+      <c r="B121" s="14" t="inlineStr">
         <is>
           <t>Epithalon</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D119" s="8" t="inlineStr">
+      <c r="C121" s="15" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D121" s="16" t="inlineStr">
         <is>
           <t>$64</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="16" customHeight="1">
-      <c r="A120" s="5" t="inlineStr">
+    <row r="122" ht="16" customHeight="1">
+      <c r="A122" s="13" t="inlineStr">
         <is>
           <t>ET50</t>
         </is>
       </c>
-      <c r="B120" s="6" t="inlineStr">
+      <c r="B122" s="14" t="inlineStr">
         <is>
           <t>Epithalon</t>
         </is>
       </c>
-      <c r="C120" s="7" t="inlineStr">
+      <c r="C122" s="15" t="inlineStr">
         <is>
           <t>50mg</t>
         </is>
       </c>
-      <c r="D120" s="8" t="inlineStr">
+      <c r="D122" s="16" t="inlineStr">
         <is>
           <t>$240</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="16" customHeight="1">
-      <c r="A121" s="9" t="inlineStr">
+    <row r="123" ht="16" customHeight="1">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>MS10</t>
         </is>
       </c>
-      <c r="B121" s="10" t="inlineStr">
+      <c r="B123" s="18" t="inlineStr">
         <is>
           <t>MOTS-c</t>
         </is>
       </c>
-      <c r="C121" s="11" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D121" s="12" t="inlineStr">
+      <c r="C123" s="19" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D123" s="20" t="inlineStr">
         <is>
           <t>$82</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="16" customHeight="1">
-      <c r="A122" s="9" t="inlineStr">
+    <row r="124" ht="16" customHeight="1">
+      <c r="A124" s="17" t="inlineStr">
         <is>
           <t>MS20</t>
         </is>
       </c>
-      <c r="B122" s="10" t="inlineStr">
+      <c r="B124" s="18" t="inlineStr">
         <is>
           <t>MOTS-c</t>
         </is>
       </c>
-      <c r="C122" s="11" t="inlineStr">
+      <c r="C124" s="19" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D122" s="12" t="inlineStr">
+      <c r="D124" s="20" t="inlineStr">
         <is>
           <t>$112</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="16" customHeight="1">
-      <c r="A123" s="9" t="inlineStr">
+    <row r="125" ht="16" customHeight="1">
+      <c r="A125" s="17" t="inlineStr">
         <is>
           <t>MS40</t>
         </is>
       </c>
-      <c r="B123" s="10" t="inlineStr">
+      <c r="B125" s="18" t="inlineStr">
         <is>
           <t>MOTS-c</t>
         </is>
       </c>
-      <c r="C123" s="11" t="inlineStr">
+      <c r="C125" s="19" t="inlineStr">
         <is>
           <t>40mg</t>
         </is>
       </c>
-      <c r="D123" s="12" t="inlineStr">
+      <c r="D125" s="20" t="inlineStr">
         <is>
           <t>$197</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="16" customHeight="1">
-      <c r="A124" s="13" t="inlineStr">
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="21" t="inlineStr">
         <is>
           <t>TA2</t>
         </is>
       </c>
-      <c r="B124" s="14" t="inlineStr">
+      <c r="B126" s="22" t="inlineStr">
         <is>
           <t>Thymosin Alpha-1</t>
         </is>
       </c>
-      <c r="C124" s="15" t="inlineStr">
+      <c r="C126" s="23" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D124" s="16" t="inlineStr">
+      <c r="D126" s="24" t="inlineStr">
         <is>
           <t>$73</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="16" customHeight="1">
-      <c r="A125" s="13" t="inlineStr">
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="21" t="inlineStr">
         <is>
           <t>TA5</t>
         </is>
       </c>
-      <c r="B125" s="14" t="inlineStr">
+      <c r="B127" s="22" t="inlineStr">
         <is>
           <t>Thymosin Alpha-1</t>
         </is>
       </c>
-      <c r="C125" s="15" t="inlineStr">
+      <c r="C127" s="23" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D127" s="24" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="16" customHeight="1">
-      <c r="A126" s="13" t="inlineStr">
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="21" t="inlineStr">
         <is>
           <t>TA10</t>
         </is>
       </c>
-      <c r="B126" s="14" t="inlineStr">
+      <c r="B128" s="22" t="inlineStr">
         <is>
           <t>Thymosin Alpha-1</t>
         </is>
       </c>
-      <c r="C126" s="15" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D126" s="16" t="inlineStr">
+      <c r="C128" s="23" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D128" s="24" t="inlineStr">
         <is>
           <t>$176</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="16" customHeight="1">
-      <c r="A127" s="17" t="inlineStr">
+    <row r="129" ht="16" customHeight="1">
+      <c r="A129" s="25" t="inlineStr">
         <is>
           <t>5AM</t>
         </is>
       </c>
-      <c r="B127" s="18" t="inlineStr">
+      <c r="B129" s="26" t="inlineStr">
         <is>
           <t>5-Amino/MQ</t>
         </is>
       </c>
-      <c r="C127" s="19" t="inlineStr">
+      <c r="C129" s="27" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D127" s="20" t="inlineStr">
+      <c r="D129" s="28" t="inlineStr">
         <is>
           <t>$183</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="16" customHeight="1">
-      <c r="A128" s="17" t="inlineStr">
+    <row r="130" ht="16" customHeight="1">
+      <c r="A130" s="25" t="inlineStr">
         <is>
           <t>5AM10</t>
         </is>
       </c>
-      <c r="B128" s="18" t="inlineStr">
+      <c r="B130" s="26" t="inlineStr">
         <is>
           <t>5-Amino/MQ</t>
         </is>
       </c>
-      <c r="C128" s="19" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D128" s="20" t="inlineStr">
+      <c r="C130" s="27" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D130" s="28" t="inlineStr">
         <is>
           <t>$261</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="16" customHeight="1">
-      <c r="A129" s="17" t="inlineStr">
+    <row r="131" ht="16" customHeight="1">
+      <c r="A131" s="25" t="inlineStr">
         <is>
           <t>50AM</t>
         </is>
       </c>
-      <c r="B129" s="18" t="inlineStr">
+      <c r="B131" s="26" t="inlineStr">
         <is>
           <t>5-Amino/MQ</t>
         </is>
       </c>
-      <c r="C129" s="19" t="inlineStr">
+      <c r="C131" s="27" t="inlineStr">
         <is>
           <t>50mg</t>
         </is>
       </c>
-      <c r="D129" s="20" t="inlineStr">
+      <c r="D131" s="28" t="inlineStr">
         <is>
           <t>$812</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="16" customHeight="1">
-      <c r="A130" s="21" t="inlineStr">
+    <row r="132" ht="16" customHeight="1">
+      <c r="A132" s="29" t="inlineStr">
         <is>
           <t>SK5</t>
         </is>
       </c>
-      <c r="B130" s="22" t="inlineStr">
+      <c r="B132" s="30" t="inlineStr">
         <is>
           <t>Selank</t>
         </is>
       </c>
-      <c r="C130" s="23" t="inlineStr">
+      <c r="C132" s="31" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D130" s="24" t="inlineStr">
+      <c r="D132" s="32" t="inlineStr">
         <is>
           <t>$55</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="16" customHeight="1">
-      <c r="A131" s="21" t="inlineStr">
+    <row r="133" ht="16" customHeight="1">
+      <c r="A133" s="29" t="inlineStr">
         <is>
           <t>SK10</t>
         </is>
       </c>
-      <c r="B131" s="22" t="inlineStr">
+      <c r="B133" s="30" t="inlineStr">
         <is>
           <t>Selank</t>
         </is>
       </c>
-      <c r="C131" s="23" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D131" s="24" t="inlineStr">
+      <c r="C133" s="31" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D133" s="32" t="inlineStr">
         <is>
           <t>$92</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="16" customHeight="1">
-      <c r="A132" s="25" t="inlineStr">
+    <row r="134" ht="16" customHeight="1">
+      <c r="A134" s="33" t="inlineStr">
         <is>
           <t>XA5</t>
         </is>
       </c>
-      <c r="B132" s="26" t="inlineStr">
+      <c r="B134" s="34" t="inlineStr">
         <is>
           <t>Semax</t>
         </is>
       </c>
-      <c r="C132" s="27" t="inlineStr">
+      <c r="C134" s="35" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D132" s="28" t="inlineStr">
+      <c r="D134" s="36" t="inlineStr">
         <is>
           <t>$53</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="16" customHeight="1">
-      <c r="A133" s="25" t="inlineStr">
+    <row r="135" ht="16" customHeight="1">
+      <c r="A135" s="33" t="inlineStr">
         <is>
           <t>XA10</t>
         </is>
       </c>
-      <c r="B133" s="26" t="inlineStr">
+      <c r="B135" s="34" t="inlineStr">
         <is>
           <t>Semax</t>
         </is>
       </c>
-      <c r="C133" s="27" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D133" s="28" t="inlineStr">
+      <c r="C135" s="35" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D135" s="36" t="inlineStr">
         <is>
           <t>$92</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="16" customHeight="1">
-      <c r="A134" s="29" t="inlineStr">
+    <row r="136" ht="16" customHeight="1">
+      <c r="A136" s="37" t="inlineStr">
         <is>
           <t>DS2</t>
         </is>
       </c>
-      <c r="B134" s="30" t="inlineStr">
+      <c r="B136" s="38" t="inlineStr">
         <is>
           <t>DSIP</t>
         </is>
       </c>
-      <c r="C134" s="31" t="inlineStr">
+      <c r="C136" s="39" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D134" s="32" t="inlineStr">
+      <c r="D136" s="40" t="inlineStr">
         <is>
           <t>$38</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="16" customHeight="1">
-      <c r="A135" s="29" t="inlineStr">
+    <row r="137" ht="16" customHeight="1">
+      <c r="A137" s="37" t="inlineStr">
         <is>
           <t>DS5</t>
         </is>
       </c>
-      <c r="B135" s="30" t="inlineStr">
+      <c r="B137" s="38" t="inlineStr">
         <is>
           <t>DSIP</t>
         </is>
       </c>
-      <c r="C135" s="31" t="inlineStr">
+      <c r="C137" s="39" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D135" s="32" t="inlineStr">
+      <c r="D137" s="40" t="inlineStr">
         <is>
           <t>$58</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="16" customHeight="1">
-      <c r="A136" s="29" t="inlineStr">
+    <row r="138" ht="16" customHeight="1">
+      <c r="A138" s="37" t="inlineStr">
         <is>
           <t>DS10</t>
         </is>
       </c>
-      <c r="B136" s="30" t="inlineStr">
+      <c r="B138" s="38" t="inlineStr">
         <is>
           <t>DSIP</t>
         </is>
       </c>
-      <c r="C136" s="31" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D136" s="32" t="inlineStr">
+      <c r="C138" s="39" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D138" s="40" t="inlineStr">
         <is>
           <t>$104</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="16" customHeight="1">
-      <c r="A137" s="33" t="inlineStr">
+    <row r="139" ht="16" customHeight="1">
+      <c r="A139" s="41" t="inlineStr">
         <is>
           <t>PI5</t>
         </is>
       </c>
-      <c r="B137" s="34" t="inlineStr">
+      <c r="B139" s="42" t="inlineStr">
         <is>
           <t>Pinealon</t>
         </is>
       </c>
-      <c r="C137" s="35" t="inlineStr">
+      <c r="C139" s="43" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D137" s="36" t="inlineStr">
+      <c r="D139" s="44" t="inlineStr">
         <is>
           <t>$75</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="16" customHeight="1">
-      <c r="A138" s="33" t="inlineStr">
-        <is>
-          <t>PI10</t>
-        </is>
-      </c>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>Pinealon</t>
-        </is>
-      </c>
-      <c r="C138" s="35" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D138" s="36" t="inlineStr">
-        <is>
-          <t>$125</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="16" customHeight="1">
-      <c r="A139" s="37" t="inlineStr">
-        <is>
-          <t>MEL10</t>
-        </is>
-      </c>
-      <c r="B139" s="38" t="inlineStr">
-        <is>
-          <t>Melatonin</t>
-        </is>
-      </c>
-      <c r="C139" s="39" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D139" s="40" t="inlineStr">
-        <is>
-          <t>$133</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="41" t="inlineStr">
         <is>
+          <t>PI10</t>
+        </is>
+      </c>
+      <c r="B140" s="42" t="inlineStr">
+        <is>
+          <t>Pinealon</t>
+        </is>
+      </c>
+      <c r="C140" s="43" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D140" s="44" t="inlineStr">
+        <is>
+          <t>$125</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="16" customHeight="1">
+      <c r="A141" s="45" t="inlineStr">
+        <is>
+          <t>MEL10</t>
+        </is>
+      </c>
+      <c r="B141" s="46" t="inlineStr">
+        <is>
+          <t>Melatonin</t>
+        </is>
+      </c>
+      <c r="C141" s="47" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D141" s="48" t="inlineStr">
+        <is>
+          <t>$133</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="16" customHeight="1">
+      <c r="A142" s="49" t="inlineStr">
+        <is>
           <t>OT2</t>
         </is>
       </c>
-      <c r="B140" s="42" t="inlineStr">
+      <c r="B142" s="50" t="inlineStr">
         <is>
           <t>Oxytocin</t>
         </is>
       </c>
-      <c r="C140" s="43" t="inlineStr">
+      <c r="C142" s="51" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D140" s="44" t="inlineStr">
+      <c r="D142" s="52" t="inlineStr">
         <is>
           <t>$72</t>
         </is>
       </c>
     </row>
-    <row r="141" ht="16" customHeight="1">
-      <c r="A141" s="41" t="inlineStr">
+    <row r="143" ht="16" customHeight="1">
+      <c r="A143" s="49" t="inlineStr">
         <is>
           <t>OT5</t>
         </is>
       </c>
-      <c r="B141" s="42" t="inlineStr">
+      <c r="B143" s="50" t="inlineStr">
         <is>
           <t>Oxytocin</t>
         </is>
       </c>
-      <c r="C141" s="43" t="inlineStr">
+      <c r="C143" s="51" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D141" s="44" t="inlineStr">
+      <c r="D143" s="52" t="inlineStr">
         <is>
           <t>$125</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="16" customHeight="1">
-      <c r="A142" s="41" t="inlineStr">
-        <is>
-          <t>OT10</t>
-        </is>
-      </c>
-      <c r="B142" s="42" t="inlineStr">
-        <is>
-          <t>Oxytocin</t>
-        </is>
-      </c>
-      <c r="C142" s="43" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D142" s="44" t="inlineStr">
-        <is>
-          <t>$232</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="16" customHeight="1">
-      <c r="A143" s="45" t="inlineStr">
-        <is>
-          <t>AR50</t>
-        </is>
-      </c>
-      <c r="B143" s="46" t="inlineStr">
-        <is>
-          <t>AICAR</t>
-        </is>
-      </c>
-      <c r="C143" s="47" t="inlineStr">
-        <is>
-          <t>50mg</t>
-        </is>
-      </c>
-      <c r="D143" s="48" t="inlineStr">
-        <is>
-          <t>$80</t>
         </is>
       </c>
     </row>
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="49" t="inlineStr">
         <is>
+          <t>OT10</t>
+        </is>
+      </c>
+      <c r="B144" s="50" t="inlineStr">
+        <is>
+          <t>Oxytocin</t>
+        </is>
+      </c>
+      <c r="C144" s="51" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D144" s="52" t="inlineStr">
+        <is>
+          <t>$232</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="16" customHeight="1">
+      <c r="A145" s="53" t="inlineStr">
+        <is>
+          <t>AR50</t>
+        </is>
+      </c>
+      <c r="B145" s="54" t="inlineStr">
+        <is>
+          <t>AICAR</t>
+        </is>
+      </c>
+      <c r="C145" s="55" t="inlineStr">
+        <is>
+          <t>50mg</t>
+        </is>
+      </c>
+      <c r="D145" s="56" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="16" customHeight="1">
+      <c r="A146" s="57" t="inlineStr">
+        <is>
           <t>2S10</t>
         </is>
       </c>
-      <c r="B144" s="50" t="inlineStr">
+      <c r="B146" s="58" t="inlineStr">
         <is>
           <t>SS-31</t>
         </is>
       </c>
-      <c r="C144" s="51" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D144" s="52" t="inlineStr">
+      <c r="C146" s="59" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D146" s="60" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="16" customHeight="1">
-      <c r="A145" s="49" t="inlineStr">
+    <row r="147" ht="16" customHeight="1">
+      <c r="A147" s="57" t="inlineStr">
         <is>
           <t>2S50</t>
         </is>
       </c>
-      <c r="B145" s="50" t="inlineStr">
+      <c r="B147" s="58" t="inlineStr">
         <is>
           <t>SS-31</t>
         </is>
       </c>
-      <c r="C145" s="51" t="inlineStr">
+      <c r="C147" s="59" t="inlineStr">
         <is>
           <t>50mg</t>
         </is>
       </c>
-      <c r="D145" s="52" t="inlineStr">
+      <c r="D147" s="60" t="inlineStr">
         <is>
           <t>$414</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="16" customHeight="1">
-      <c r="A146" s="53" t="inlineStr">
+    <row r="148" ht="16" customHeight="1">
+      <c r="A148" s="61" t="inlineStr">
         <is>
           <t>ADA5</t>
         </is>
       </c>
-      <c r="B146" s="54" t="inlineStr">
+      <c r="B148" s="62" t="inlineStr">
         <is>
           <t>Admax</t>
         </is>
       </c>
-      <c r="C146" s="55" t="inlineStr">
+      <c r="C148" s="63" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D146" s="56" t="inlineStr">
+      <c r="D148" s="64" t="inlineStr">
         <is>
           <t>$158</t>
         </is>
       </c>
     </row>
-    <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="53" t="inlineStr">
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="61" t="inlineStr">
         <is>
           <t>ADA10</t>
         </is>
       </c>
-      <c r="B147" s="54" t="inlineStr">
+      <c r="B149" s="62" t="inlineStr">
         <is>
           <t>Admax</t>
         </is>
       </c>
-      <c r="C147" s="55" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D147" s="56" t="inlineStr">
+      <c r="C149" s="63" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D149" s="64" t="inlineStr">
         <is>
           <t>$265</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="16" customHeight="1">
-      <c r="A148" s="57" t="inlineStr">
+    <row r="150" ht="16" customHeight="1">
+      <c r="A150" s="65" t="inlineStr">
         <is>
           <t>F42</t>
         </is>
       </c>
-      <c r="B148" s="58" t="inlineStr">
+      <c r="B150" s="66" t="inlineStr">
         <is>
           <t>FOXO4-DRI</t>
         </is>
       </c>
-      <c r="C148" s="59" t="inlineStr">
+      <c r="C150" s="67" t="inlineStr">
         <is>
           <t>2mg</t>
         </is>
       </c>
-      <c r="D148" s="60" t="inlineStr">
+      <c r="D150" s="68" t="inlineStr">
         <is>
           <t>$232</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="57" t="inlineStr">
+    <row r="151" ht="16" customHeight="1">
+      <c r="A151" s="65" t="inlineStr">
         <is>
           <t>F45</t>
         </is>
       </c>
-      <c r="B149" s="58" t="inlineStr">
+      <c r="B151" s="66" t="inlineStr">
         <is>
           <t>FOXO4-DRI</t>
         </is>
       </c>
-      <c r="C149" s="59" t="inlineStr">
+      <c r="C151" s="67" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D149" s="60" t="inlineStr">
+      <c r="D151" s="68" t="inlineStr">
         <is>
           <t>$373</t>
         </is>
       </c>
     </row>
-    <row r="150" ht="16" customHeight="1">
-      <c r="A150" s="57" t="inlineStr">
+    <row r="152" ht="16" customHeight="1">
+      <c r="A152" s="65" t="inlineStr">
         <is>
           <t>F410</t>
         </is>
       </c>
-      <c r="B150" s="58" t="inlineStr">
+      <c r="B152" s="66" t="inlineStr">
         <is>
           <t>FOXO4-DRI</t>
         </is>
       </c>
-      <c r="C150" s="59" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D150" s="60" t="inlineStr">
+      <c r="C152" s="67" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D152" s="68" t="inlineStr">
         <is>
           <t>$629</t>
         </is>
       </c>
     </row>
-    <row r="151" ht="16" customHeight="1">
-      <c r="A151" s="61" t="inlineStr">
+    <row r="153" ht="16" customHeight="1">
+      <c r="A153" s="5" t="inlineStr">
         <is>
           <t>CAR10</t>
         </is>
       </c>
-      <c r="B151" s="62" t="inlineStr">
+      <c r="B153" s="6" t="inlineStr">
         <is>
           <t>Cardiogen</t>
         </is>
       </c>
-      <c r="C151" s="63" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D151" s="64" t="inlineStr">
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
         <is>
           <t>$174</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="16" customHeight="1">
-      <c r="A152" s="61" t="inlineStr">
+    <row r="154" ht="16" customHeight="1">
+      <c r="A154" s="5" t="inlineStr">
         <is>
           <t>CAR20</t>
         </is>
       </c>
-      <c r="B152" s="62" t="inlineStr">
+      <c r="B154" s="6" t="inlineStr">
         <is>
           <t>Cardiogen</t>
         </is>
       </c>
-      <c r="C152" s="63" t="inlineStr">
+      <c r="C154" s="7" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D152" s="64" t="inlineStr">
+      <c r="D154" s="8" t="inlineStr">
         <is>
           <t>$298</t>
         </is>
       </c>
     </row>
-    <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="65" t="inlineStr">
+    <row r="155" ht="16" customHeight="1">
+      <c r="A155" s="9" t="inlineStr">
         <is>
           <t>CART10</t>
         </is>
       </c>
-      <c r="B153" s="66" t="inlineStr">
+      <c r="B155" s="10" t="inlineStr">
         <is>
           <t>Cartalax</t>
         </is>
       </c>
-      <c r="C153" s="67" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D153" s="68" t="inlineStr">
+      <c r="C155" s="11" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D155" s="12" t="inlineStr">
         <is>
           <t>$191</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="65" t="inlineStr">
+    <row r="156" ht="16" customHeight="1">
+      <c r="A156" s="9" t="inlineStr">
         <is>
           <t>CART20</t>
         </is>
       </c>
-      <c r="B154" s="66" t="inlineStr">
+      <c r="B156" s="10" t="inlineStr">
         <is>
           <t>Cartalax</t>
         </is>
       </c>
-      <c r="C154" s="67" t="inlineStr">
+      <c r="C156" s="11" t="inlineStr">
         <is>
           <t>20mg</t>
         </is>
       </c>
-      <c r="D154" s="68" t="inlineStr">
+      <c r="D156" s="12" t="inlineStr">
         <is>
           <t>$323</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="16" customHeight="1">
-      <c r="A155" s="5" t="inlineStr">
+    <row r="157" ht="16" customHeight="1">
+      <c r="A157" s="13" t="inlineStr">
         <is>
           <t>CRY10</t>
         </is>
       </c>
-      <c r="B155" s="6" t="inlineStr">
+      <c r="B157" s="14" t="inlineStr">
         <is>
           <t>Crystagen</t>
         </is>
       </c>
-      <c r="C155" s="7" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D155" s="8" t="inlineStr">
+      <c r="C157" s="15" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D157" s="16" t="inlineStr">
         <is>
           <t>$158</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="16" customHeight="1">
-      <c r="A156" s="5" t="inlineStr">
-        <is>
-          <t>CRY20</t>
-        </is>
-      </c>
-      <c r="B156" s="6" t="inlineStr">
-        <is>
-          <t>Crystagen</t>
-        </is>
-      </c>
-      <c r="C156" s="7" t="inlineStr">
-        <is>
-          <t>20mg</t>
-        </is>
-      </c>
-      <c r="D156" s="8" t="inlineStr">
-        <is>
-          <t>$290</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="16" customHeight="1">
-      <c r="A157" s="9" t="inlineStr">
-        <is>
-          <t>HUM10</t>
-        </is>
-      </c>
-      <c r="B157" s="10" t="inlineStr">
-        <is>
-          <t>Humanin</t>
-        </is>
-      </c>
-      <c r="C157" s="11" t="inlineStr">
-        <is>
-          <t>10mg</t>
-        </is>
-      </c>
-      <c r="D157" s="12" t="inlineStr">
-        <is>
-          <t>$737</t>
         </is>
       </c>
     </row>
     <row r="158" ht="16" customHeight="1">
       <c r="A158" s="13" t="inlineStr">
         <is>
-          <t>MAT10</t>
+          <t>CRY20</t>
         </is>
       </c>
       <c r="B158" s="14" t="inlineStr">
         <is>
-          <t>Matrixyl</t>
+          <t>Crystagen</t>
         </is>
       </c>
       <c r="C158" s="15" t="inlineStr">
         <is>
-          <t>10mg</t>
+          <t>20mg</t>
         </is>
       </c>
       <c r="D158" s="16" t="inlineStr">
         <is>
-          <t>$82</t>
+          <t>$290</t>
         </is>
       </c>
     </row>
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="17" t="inlineStr">
         <is>
-          <t>PN5</t>
+          <t>HUM10</t>
         </is>
       </c>
       <c r="B159" s="18" t="inlineStr">
         <is>
-          <t>PNC-27</t>
+          <t>Humanin</t>
         </is>
       </c>
       <c r="C159" s="19" t="inlineStr">
         <is>
-          <t>5mg</t>
+          <t>10mg</t>
         </is>
       </c>
       <c r="D159" s="20" t="inlineStr">
         <is>
-          <t>$290</t>
+          <t>$737</t>
         </is>
       </c>
     </row>
     <row r="160" ht="16" customHeight="1">
       <c r="A160" s="21" t="inlineStr">
         <is>
+          <t>MAT10</t>
+        </is>
+      </c>
+      <c r="B160" s="22" t="inlineStr">
+        <is>
+          <t>Matrixyl</t>
+        </is>
+      </c>
+      <c r="C160" s="23" t="inlineStr">
+        <is>
+          <t>10mg</t>
+        </is>
+      </c>
+      <c r="D160" s="24" t="inlineStr">
+        <is>
+          <t>$82</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="16" customHeight="1">
+      <c r="A161" s="25" t="inlineStr">
+        <is>
+          <t>PN5</t>
+        </is>
+      </c>
+      <c r="B161" s="26" t="inlineStr">
+        <is>
+          <t>PNC-27</t>
+        </is>
+      </c>
+      <c r="C161" s="27" t="inlineStr">
+        <is>
+          <t>5mg</t>
+        </is>
+      </c>
+      <c r="D161" s="28" t="inlineStr">
+        <is>
+          <t>$290</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="16" customHeight="1">
+      <c r="A162" s="29" t="inlineStr">
+        <is>
           <t>SLU5</t>
         </is>
       </c>
-      <c r="B160" s="22" t="inlineStr">
+      <c r="B162" s="30" t="inlineStr">
         <is>
           <t>SLU-PP-322</t>
         </is>
       </c>
-      <c r="C160" s="23" t="inlineStr">
+      <c r="C162" s="31" t="inlineStr">
         <is>
           <t>5mg</t>
         </is>
       </c>
-      <c r="D160" s="24" t="inlineStr">
+      <c r="D162" s="32" t="inlineStr">
         <is>
           <t>$216</t>
         </is>
       </c>
     </row>
-    <row r="161" ht="16" customHeight="1">
-      <c r="A161" s="69" t="inlineStr">
+    <row r="163" ht="16" customHeight="1">
+      <c r="A163" s="69" t="inlineStr">
         <is>
           <t>所有产品仅供研究使用 · 最低订购: 1套 · 价格可能变动  |  Research use only · Min order: 1 kit · Prices subject to change</t>
         </is>
@@ -4210,11 +4254,11 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A112:D112"/>
+    <mergeCell ref="A163:D163"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A161:D161"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NAD+ pricing: smooth curve mirroring catalog (100mg $100 / 500mg $405 / 1000mg $740)
Replaces the broken $100/$240/$260 (where 1000mg was only +$20 over 500mg). Now follows
the catalog's ~mg^0.87 curve, premium-anchored at $1.00/mg. Sheet + catalog updated, xlsx
regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/price_list.xlsx
+++ b/static/price_list.xlsx
@@ -3228,7 +3228,7 @@
       </c>
       <c r="D116" s="8" t="inlineStr">
         <is>
-          <t>$240</t>
+          <t>$405</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>$260</t>
+          <t>$740</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NAD+ competitive pricing $55/$135/$195 + dedupe catalog NAD rows
- NAD+ set to competitive loss-leader prices (3.1-4.1x cost) per manual decision;
  other sellers are cheaper, not a margin product.
- Removed a duplicate NAD catalog block; kept one with real internal costs
  (17.73/42.84/47.27) so the 3x floor sits below the new prices (no guardrail override).
- Sheet regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/price_list.xlsx
+++ b/static/price_list.xlsx
@@ -3206,7 +3206,7 @@
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$55</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="D116" s="8" t="inlineStr">
         <is>
-          <t>$405</t>
+          <t>$135</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>$740</t>
+          <t>$195</t>
         </is>
       </c>
     </row>

</xml_diff>